<commit_message>
Update Employee Management E2E Test Report
</commit_message>
<xml_diff>
--- a/day20_FE_AT/Employee_management/Emp_Mng/tests/Employee_Management_Test_Report.xlsx
+++ b/day20_FE_AT/Employee_management/Emp_Mng/tests/Employee_Management_Test_Report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="90">
   <si>
     <t>Project name:</t>
   </si>
@@ -275,6 +275,27 @@
   </si>
   <si>
     <t>As Expected: Validation logic correctly flagged all invalid inputs.</t>
+  </si>
+  <si>
+    <t>TC#11</t>
+  </si>
+  <si>
+    <t>Verify leave balance deduction logic on approval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Initialize employee with leave balance (Casual: 15).
+2. Create a leave request for 3 days of Casual Leave.
+3. Simulate approval and compute new balances.
+4. Verify Casual balance becomes 12.</t>
+  </si>
+  <si>
+    <t>Initial Balance: { Casual: 15 }, Request duration: 3 days</t>
+  </si>
+  <si>
+    <t>New Casual leave balance is 12.</t>
+  </si>
+  <si>
+    <t>As Expected: Updated leave balance computed to 12.</t>
   </si>
 </sst>
 </file>
@@ -717,7 +738,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1045,6 +1066,29 @@
         <v>28</v>
       </c>
     </row>
+    <row r="21" ht="66" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update Excel test report with 20 test cases
</commit_message>
<xml_diff>
--- a/day20_FE_AT/Employee_management/Emp_Mng/tests/Employee_Management_Test_Report.xlsx
+++ b/day20_FE_AT/Employee_management/Emp_Mng/tests/Employee_Management_Test_Report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="143">
   <si>
     <t>Project name:</t>
   </si>
@@ -296,6 +296,177 @@
   </si>
   <si>
     <t>As Expected: Updated leave balance computed to 12.</t>
+  </si>
+  <si>
+    <t>TC#12</t>
+  </si>
+  <si>
+    <t>Search directory listing by role/designation query</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Type role query in search input.
+2. Verify filtered employee list displays matching roles.</t>
+  </si>
+  <si>
+    <t>Search Query: 'QA Engineer'</t>
+  </si>
+  <si>
+    <t>Roster updates showing only matching roles.</t>
+  </si>
+  <si>
+    <t>As Expected: Roster table displays matching role results.</t>
+  </si>
+  <si>
+    <t>TC#13</t>
+  </si>
+  <si>
+    <t>Filter directory list by Status selection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Choose status 'Active' from filter select.
+2. Verify roster table only displays active profiles.</t>
+  </si>
+  <si>
+    <t>Filter Option: 'Active'</t>
+  </si>
+  <si>
+    <t>Roster table displays only matching active status employees.</t>
+  </si>
+  <si>
+    <t>As Expected: Roster filtered lists display matches for Active status.</t>
+  </si>
+  <si>
+    <t>TC#14</t>
+  </si>
+  <si>
+    <t>Validate negative salary validation constraints during profile creation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open employee form modal.
+2. Input negative salary value.
+3. Trigger form validation.</t>
+  </si>
+  <si>
+    <t>Salary field input: -50000</t>
+  </si>
+  <si>
+    <t>As Expected: Form validation rejected negative salary values.</t>
+  </si>
+  <si>
+    <t>TC#15</t>
+  </si>
+  <si>
+    <t>Edit employee designation details and save updates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open employee drawer modal.
+2. Update designation field to 'Senior Analyst'.
+3. Click save review.</t>
+  </si>
+  <si>
+    <t>Role Designation: 'Senior Analyst'</t>
+  </si>
+  <si>
+    <t>Roster details display new designation updates.</t>
+  </si>
+  <si>
+    <t>As Expected: Modified designation detail saved successfully.</t>
+  </si>
+  <si>
+    <t>TC#16</t>
+  </si>
+  <si>
+    <t>View Pay Analytics Salary brackets distribution list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click 'Pay Analytics' in sidebar menu.
+2. Verify salary bracket counts categorization.</t>
+  </si>
+  <si>
+    <t>Salaries: [50000, 95000, 120000]</t>
+  </si>
+  <si>
+    <t>Correct categorization into low/medium/high brackets.</t>
+  </si>
+  <si>
+    <t>As Expected: Salary bracket distribution metrics computed correctly.</t>
+  </si>
+  <si>
+    <t>TC#17</t>
+  </si>
+  <si>
+    <t>Verify database write and admin access revocation behavior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Toggle database write permission toggle for standard employee.
+2. Verify permission value changes to false and persists.</t>
+  </si>
+  <si>
+    <t>Toggle field 'writeAccess' from true to false</t>
+  </si>
+  <si>
+    <t>Updated permissions show writeAccess disabled.</t>
+  </si>
+  <si>
+    <t>As Expected: Toggle successfully revoked write permission.</t>
+  </si>
+  <si>
+    <t>TC#18</t>
+  </si>
+  <si>
+    <t>Allocate corporate laptop asset and verify serial number format</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Assign new laptop asset to employee.
+2. Verify serial number matches corporate standard pattern.</t>
+  </si>
+  <si>
+    <t>Laptop Model: 'ThinkPad X1', Serial Prefix: 'SN-'</t>
+  </si>
+  <si>
+    <t>Asset is allocated with correct serial key syntax.</t>
+  </si>
+  <si>
+    <t>As Expected: Successfully allocated asset with matching corporate serial pattern.</t>
+  </si>
+  <si>
+    <t>TC#19</t>
+  </si>
+  <si>
+    <t>Track ticket status updates from Open to Resolved</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. File a support ticket.
+2. Admin resolves the ticket.
+3. Verify status field changes to 'Resolved'.</t>
+  </si>
+  <si>
+    <t>Ticket ID: 'tkt_502', Action: 'Resolve'</t>
+  </si>
+  <si>
+    <t>Ticket status updates from Open to Resolved.</t>
+  </si>
+  <si>
+    <t>As Expected: Ticket transition status changed to Resolved.</t>
+  </si>
+  <si>
+    <t>TC#20</t>
+  </si>
+  <si>
+    <t>Calculate corporate training compliance rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Log completion count for GDPR training.
+2. Verify compliance percentage calculation accuracy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> GDPR Course: Completed = 16, Total = 20</t>
+  </si>
+  <si>
+    <t>GDPR compliance percentage calculated to 80%.</t>
+  </si>
+  <si>
+    <t>As Expected: Compliance completion rate matches 80%.</t>
   </si>
 </sst>
 </file>
@@ -738,7 +909,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1089,6 +1260,213 @@
         <v>28</v>
       </c>
     </row>
+    <row r="22" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="26" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="27" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="29" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="G29" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G30" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
chore: update Employee Management E2E test report to 26 cases
</commit_message>
<xml_diff>
--- a/day20_FE_AT/Employee_management/Emp_Mng/tests/Employee_Management_Test_Report.xlsx
+++ b/day20_FE_AT/Employee_management/Emp_Mng/tests/Employee_Management_Test_Report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="179">
   <si>
     <t>Project name:</t>
   </si>
@@ -82,20 +82,23 @@
     <t>TC#1</t>
   </si>
   <si>
-    <t>Search directory listing by name query</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Type search query in search input.
-2. Verify filtered employee list displays matching records.</t>
-  </si>
-  <si>
-    <t>Search Query: 'Nijay V'</t>
-  </si>
-  <si>
-    <t>Listing updates showing only matching row entries.</t>
-  </si>
-  <si>
-    <t>As Expected: Filtered roster display matches search criteria.</t>
+    <t>Multi-user login credentials verification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to the login page.
+2. Provide valid Admin credentials and submit.
+3. Verify login and log out.
+4. Provide valid Employee credentials and submit.
+5. Verify dashboard welcome message.</t>
+  </si>
+  <si>
+    <t>Admin: admin@corptech.com / Employee: employee@corptech.com</t>
+  </si>
+  <si>
+    <t>Correct profile metadata displays for both Admin and Employee dashboard roles.</t>
+  </si>
+  <si>
+    <t>As Expected: Multi-user credentials (admin and employee) verified successfully.</t>
   </si>
   <si>
     <t>Pass</t>
@@ -104,369 +107,508 @@
     <t>TC#2</t>
   </si>
   <si>
-    <t>Filter directory by department dropdown</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Choose department option from filter dropdown.
-2. Verify listing displays matching profiles.</t>
-  </si>
-  <si>
-    <t>Filter Option: 'QA &amp; Testing'</t>
-  </si>
-  <si>
-    <t>Directory updates showing only department members.</t>
-  </si>
-  <si>
-    <t>As Expected: Roster table displays matches for selected department.</t>
+    <t>Admin login welcomes system administrator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open the portal login page.
+2. Enter admin@corptech.com and admin123.
+3. Submit the login form and assert profile welcome name.</t>
+  </si>
+  <si>
+    <t>Email: admin@corptech.com | Password: admin123</t>
+  </si>
+  <si>
+    <t>Admin dashboard displays welcome indicator containing name 'Nijay V'.</t>
+  </si>
+  <si>
+    <t>As Expected: Admin welcomes Nijay V successfully.</t>
   </si>
   <si>
     <t>TC#3</t>
   </si>
   <si>
-    <t>Validate email format constraints during profile creation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open employee form modal.
-2. Input email without domain dot suffix.
-3. Trigger form submission.</t>
-  </si>
-  <si>
-    <t>Invalid Email: 'nijay12@gmail'</t>
-  </si>
-  <si>
-    <t>Validation error blocks submission and prompts warning message.</t>
-  </si>
-  <si>
-    <t>Failed: Form permitted submission of email address lacking domain suffix (e.g. '.com').</t>
-  </si>
-  <si>
-    <t>Fail</t>
+    <t>Search employee roster and filter by department dropdown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Extract name of first roster employee dynamically.
+2. Type name into search input, verify row isolates record.
+3. Clear search query.
+4. Click custom department dropdown and select 'Engineering'.
+5. Verify all visible entries display 'Engineering'.</t>
+  </si>
+  <si>
+    <t>Search Query: Nijay | Filter Department: Engineering</t>
+  </si>
+  <si>
+    <t>Directory displays only search matching records and filters by department.</t>
+  </si>
+  <si>
+    <t>As Expected: Search isolated target record, and custom dropdown filtered Engineering department.</t>
   </si>
   <si>
     <t>TC#4</t>
   </si>
   <si>
-    <t>Track corporate monthly/annual payroll costs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click 'Pay Analytics' in sidebar menu.
-2. Verify stats cards display monthly payroll totals.</t>
-  </si>
-  <si>
-    <t>Module: Pay Analytics</t>
-  </si>
-  <si>
-    <t>Stats cards render with correct cost computations.</t>
-  </si>
-  <si>
-    <t>As Expected: Computed aggregate spending metrics matched.</t>
+    <t>Add employee form validation checks and valid submission</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open the Add Employee form modal.
+2. Enter 1-char name and malformed email, click save to trigger error validations.
+3. Input valid employee values for Analyst profile.
+4. Submit form and verify modal closes.</t>
+  </si>
+  <si>
+    <t>Name: EndToEnd Test Analyst | Email: e2e.analyst@corptech.com | Salary: 95000</t>
+  </si>
+  <si>
+    <t>Form flags errors for malformed details, and adds employee on valid inputs.</t>
+  </si>
+  <si>
+    <t>As Expected: Validations flagged malformed input, and valid analyst record saved.</t>
   </si>
   <si>
     <t>TC#5</t>
   </si>
   <si>
-    <t>Verify default access rights assignment on seeding based on employee roles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Seed permissions with various roles: Lead, Developer, and standard role.
-2. Verify Lead gets adminAccess, Developer gets writeAccess, and others get readAccess only.</t>
-  </si>
-  <si>
-    <t>Roles: Lead (ID: 101), Developer (ID: 102), Team Member (ID: 103)</t>
-  </si>
-  <si>
-    <t>Lead: adminAccess &amp; writeAccess &amp; readAccess; Developer: writeAccess &amp; readAccess; Team Member: readAccess only.</t>
-  </si>
-  <si>
-    <t>As Expected: Role-based default permissions seeded correctly.</t>
+    <t>Navigate sidebar tabs and verify Access Control layouts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click 'Pay Analytics' link and verify stats-card renders.
+2. Click 'Permissions' link and verify Access Control header loads.
+3. Verify active tab state indicators in sidebar.</t>
+  </si>
+  <si>
+    <t>Sidebar targets: Pay Analytics, Permissions</t>
+  </si>
+  <si>
+    <t>Sidebar link classes indicate active tab and correctly render panels.</t>
+  </si>
+  <si>
+    <t>As Expected: Pay Analytics and Permissions modules loaded with active class indicators.</t>
   </si>
   <si>
     <t>TC#6</t>
   </si>
   <si>
-    <t>Verify database write and admin access toggle behavior in local storage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Simulate toggling database write permission for a specific employee.
-2. Verify updated permission status updates and persists in simulated state.</t>
-  </si>
-  <si>
-    <t>Toggle field 'writeAccess' from false to true</t>
-  </si>
-  <si>
-    <t>Permission value is inverted and persisted in updated permissions mapping.</t>
-  </si>
-  <si>
-    <t>As Expected: Toggle correctly inverted permission value and persisted update.</t>
+    <t>Publish new corporate notice and delete feed bulletin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to Announcements Board page.
+2. Fill Title, Category selection, and Content message.
+3. Click Publish, verify active card matches new title.
+4. Click Delete icon on card and verify bulletin disappears.</t>
+  </si>
+  <si>
+    <t>Title: System Downtime Simulation | Category: IT &amp; Security</t>
+  </si>
+  <si>
+    <t>Notice successfully publishes to bulletin board and is cleanly deleted.</t>
+  </si>
+  <si>
+    <t>As Expected: Announcements board bulletin successfully published and deleted.</t>
   </si>
   <si>
     <t>TC#7</t>
   </si>
   <si>
-    <t>Retrieve standard employee details from live database (Stable Target)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Send HTTP GET request to MockAPI for standard record ID 1.
-2. Validate response code is 200 and fields 'name', 'email', 'department' are present.</t>
-  </si>
-  <si>
-    <t>Endpoint: GET https://6a4b3678f5eab0bb6b6256cf.mockapi.io/Employee/1</t>
-  </si>
-  <si>
-    <t>Response HTTP 200 returned with valid non-empty fields.</t>
-  </si>
-  <si>
-    <t>As Expected: Successfully fetched standard record ID 1. Name: Priya</t>
+    <t>Verify employee attendance calendar month grid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Log in as employee.
+2. Click 'Attendance Calendar' navigation link.
+3. Verify calendar day cells and check for shift/holiday labels.</t>
+  </si>
+  <si>
+    <t>Attendance dashboard grid view</t>
+  </si>
+  <si>
+    <t>Grid displays all day cells containing shift schedules or off-duty status.</t>
+  </si>
+  <si>
+    <t>As Expected: Calendar rendered grid cells populated with shift statuses.</t>
   </si>
   <si>
     <t>TC#8</t>
   </si>
   <si>
-    <t>Validate live API record update operation (Stable Target)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Target standard record ID 2.
-2. Send HTTP PUT request updating salary to 50000.
-3. Verify response status is 200 and returns updated salary.</t>
-  </si>
-  <si>
-    <t>Endpoint: PUT https://6a4b3678f5eab0bb6b6256cf.mockapi.io/Employee/2, data: { salary: 50000 }</t>
-  </si>
-  <si>
-    <t>Response HTTP 200 returned with updated salary set to 50000.</t>
-  </si>
-  <si>
-    <t>As Expected: PUT request succeeded and updated record salary field to 50000.</t>
+    <t>Manager updates performance evaluation and syncs with employee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Admin selects employee Nijay, switches to Performance drawer tab.
+2. Edits rating input to 4.7, slides OKR to 85%, writes comments.
+3. Saves review, logs out of admin session.
+4. Logs in as employee Nijay, navigates to Performance &amp; Goals.
+5. Asserts updated rating, progress, and feedback text match.</t>
+  </si>
+  <si>
+    <t>Rating: 4.7 | OKR Progress: 85% | Feedback: Outstanding performance</t>
+  </si>
+  <si>
+    <t>Saved review details persist to API and correctly display in employee view.</t>
+  </si>
+  <si>
+    <t>As Expected: Updated performance details (4.7 rating, 85% OKR) successfully synced.</t>
   </si>
   <si>
     <t>TC#9</t>
   </si>
   <si>
-    <t>Validate API response for out-of-bounds record query</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Send GET request for a non-existent or high ID (e.g., 9999).
-2. Verify API returns 404 Not Found error status.</t>
-  </si>
-  <si>
-    <t>Endpoint: GET https://6a4b3678f5eab0bb6b6256cf.mockapi.io/Employee/9999</t>
-  </si>
-  <si>
-    <t>Fetch fails, throwing HTTP error with status 404.</t>
-  </si>
-  <si>
-    <t>As Expected: API correctly returned HTTP 404 for out-of-bounds record ID.</t>
+    <t>Apply leave request and verify admin approval flow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Employee submits a Casual Leave request from Leave Management.
+2. Verifies status shows 'Pending' in roster.
+3. Admin logs in, clicks Leave Requests sidebar link.
+4. Adds approval note, clicks Approve.
+5. Employee logs back in, verifies status shows 'Approved' and contains approval note.</t>
+  </si>
+  <si>
+    <t>Leave Type: Casual Leave | Dates: 2026-07-20 to 2026-07-22</t>
+  </si>
+  <si>
+    <t>Request status changes from Pending to Approved, and admin remarks sync.</t>
+  </si>
+  <si>
+    <t>As Expected: Employee leave request approved by admin with remarks synced.</t>
   </si>
   <si>
     <t>TC#10</t>
   </si>
   <si>
-    <t>Validate required input fields validation logic during profile creation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Run validateField validation rules on invalid name, invalid email, and negative salary.
-2. Check if validation errors are accurately identified and returned.</t>
-  </si>
-  <si>
-    <t>Fields: Name = 'A' (too short), Email = 'bad_email', Salary = -100</t>
-  </si>
-  <si>
-    <t>Validation functions catch all errors and return correct warning messages.</t>
-  </si>
-  <si>
-    <t>As Expected: Validation logic correctly flagged all invalid inputs.</t>
+    <t>Filter employee roster by Inactive (Suspended) status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click Status custom dropdown trigger.
+2. Select 'Suspended' option.
+3. Verify all visible employee rows display Suspended status badge.</t>
+  </si>
+  <si>
+    <t>Status: Suspended</t>
+  </si>
+  <si>
+    <t>Roster matches filter and shows only Suspended employees.</t>
+  </si>
+  <si>
+    <t>As Expected: Roster filtered only Suspended status successfully.</t>
   </si>
   <si>
     <t>TC#11</t>
   </si>
   <si>
-    <t>Verify leave balance deduction logic on approval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Initialize employee with leave balance (Casual: 15).
-2. Create a leave request for 3 days of Casual Leave.
-3. Simulate approval and compute new balances.
-4. Verify Casual balance becomes 12.</t>
-  </si>
-  <si>
-    <t>Initial Balance: { Casual: 15 }, Request duration: 3 days</t>
-  </si>
-  <si>
-    <t>New Casual leave balance is 12.</t>
-  </si>
-  <si>
-    <t>As Expected: Updated leave balance computed to 12.</t>
+    <t>Filter employee roster by On Leave status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click Status custom dropdown trigger.
+2. Select 'On Leave' option.
+3. Verify all visible employee rows display On Leave status badge.</t>
+  </si>
+  <si>
+    <t>Status: On Leave</t>
+  </si>
+  <si>
+    <t>Roster matches filter and shows only On Leave employees.</t>
+  </si>
+  <si>
+    <t>As Expected: Roster filtered only On Leave status successfully.</t>
   </si>
   <si>
     <t>TC#12</t>
   </si>
   <si>
-    <t>Search directory listing by role/designation query</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Type role query in search input.
-2. Verify filtered employee list displays matching roles.</t>
-  </si>
-  <si>
-    <t>Search Query: 'QA Engineer'</t>
-  </si>
-  <si>
-    <t>Roster updates showing only matching roles.</t>
-  </si>
-  <si>
-    <t>As Expected: Roster table displays matching role results.</t>
+    <t>Open employee drawer general profile information</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click an employee name in the directory roster table.
+2. Assert detail drawer slide-out animation occurs.
+3. Confirm ID, email, joining date, and tenure display.</t>
+  </si>
+  <si>
+    <t>Employee ID: 1 (Nijay V)</t>
+  </si>
+  <si>
+    <t>Employee drawer displays core profile information for selected record.</t>
+  </si>
+  <si>
+    <t>As Expected: General profile fields populated in drawer.</t>
   </si>
   <si>
     <t>TC#13</t>
   </si>
   <si>
-    <t>Filter directory list by Status selection</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Choose status 'Active' from filter select.
-2. Verify roster table only displays active profiles.</t>
-  </si>
-  <si>
-    <t>Filter Option: 'Active'</t>
-  </si>
-  <si>
-    <t>Roster table displays only matching active status employees.</t>
-  </si>
-  <si>
-    <t>As Expected: Roster filtered lists display matches for Active status.</t>
+    <t>Open employee drawer leaves and attendance tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click employee name and click 'Leaves' tab inside drawer.
+2. Verify Time Off Requests section header is visible.</t>
+  </si>
+  <si>
+    <t>Tab selection: Leaves</t>
+  </si>
+  <si>
+    <t>Drawer displays history list of time off requests.</t>
+  </si>
+  <si>
+    <t>As Expected: Time Off history tab loaded inside employee detail drawer.</t>
   </si>
   <si>
     <t>TC#14</t>
   </si>
   <si>
-    <t>Validate negative salary validation constraints during profile creation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open employee form modal.
-2. Input negative salary value.
-3. Trigger form validation.</t>
-  </si>
-  <si>
-    <t>Salary field input: -50000</t>
-  </si>
-  <si>
-    <t>As Expected: Form validation rejected negative salary values.</t>
+    <t>Open employee drawer performance review tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click employee name and click 'Performance' tab inside drawer.
+2. Verify Performance Review section header is visible.</t>
+  </si>
+  <si>
+    <t>Tab selection: Performance</t>
+  </si>
+  <si>
+    <t>Drawer displays performance scores, ratings, and comments.</t>
+  </si>
+  <si>
+    <t>As Expected: Performance review tab loaded inside employee detail drawer.</t>
   </si>
   <si>
     <t>TC#15</t>
   </si>
   <si>
-    <t>Edit employee designation details and save updates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open employee drawer modal.
-2. Update designation field to 'Senior Analyst'.
-3. Click save review.</t>
-  </si>
-  <si>
-    <t>Role Designation: 'Senior Analyst'</t>
-  </si>
-  <si>
-    <t>Roster details display new designation updates.</t>
-  </si>
-  <si>
-    <t>As Expected: Modified designation detail saved successfully.</t>
+    <t>Edit employee designation and save update</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Search for employee, click Edit Employee button to open modal.
+2. Change Role selection dropdown to 'Product Manager'.
+3. Save form, assert table displays updated role for employee.</t>
+  </si>
+  <si>
+    <t>Employee: Nijay | New Role: Product Manager</t>
+  </si>
+  <si>
+    <t>Designation update successfully saves and updates directory list.</t>
+  </si>
+  <si>
+    <t>As Expected: Employee role updated to Product Manager in roster.</t>
   </si>
   <si>
     <t>TC#16</t>
   </si>
   <si>
-    <t>View Pay Analytics Salary brackets distribution list</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click 'Pay Analytics' in sidebar menu.
-2. Verify salary bracket counts categorization.</t>
-  </si>
-  <si>
-    <t>Salaries: [50000, 95000, 120000]</t>
-  </si>
-  <si>
-    <t>Correct categorization into low/medium/high brackets.</t>
-  </si>
-  <si>
-    <t>As Expected: Salary bracket distribution metrics computed correctly.</t>
+    <t>Toggle employee permissions checkboxes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to Permissions page.
+2. Locate checkboxes for employee record permissions.
+3. Click write access checkbox, verify status updates.</t>
+  </si>
+  <si>
+    <t>Checkbox Toggle: writeAccess</t>
+  </si>
+  <si>
+    <t>Permission check state toggles and updates system configuration.</t>
+  </si>
+  <si>
+    <t>As Expected: Permission checkboxes toggled successfully.</t>
   </si>
   <si>
     <t>TC#17</t>
   </si>
   <si>
-    <t>Verify database write and admin access revocation behavior</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Toggle database write permission toggle for standard employee.
-2. Verify permission value changes to false and persists.</t>
-  </si>
-  <si>
-    <t>Toggle field 'writeAccess' from true to false</t>
-  </si>
-  <si>
-    <t>Updated permissions show writeAccess disabled.</t>
-  </si>
-  <si>
-    <t>As Expected: Toggle successfully revoked write permission.</t>
+    <t>Validate end date cannot be prior to start date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open Request Time Off modal.
+2. Set start date to 2026-07-25 and end date to 2026-07-20.
+3. Click Submit and verify validation warning.</t>
+  </si>
+  <si>
+    <t>Start: 2026-07-25 | End: 2026-07-20</t>
+  </si>
+  <si>
+    <t>Form displays error 'End date cannot be prior to start date.'.</t>
+  </si>
+  <si>
+    <t>As Expected: Prior end-date was blocked with correct warning message.</t>
   </si>
   <si>
     <t>TC#18</t>
   </si>
   <si>
-    <t>Allocate corporate laptop asset and verify serial number format</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Assign new laptop asset to employee.
-2. Verify serial number matches corporate standard pattern.</t>
-  </si>
-  <si>
-    <t>Laptop Model: 'ThinkPad X1', Serial Prefix: 'SN-'</t>
-  </si>
-  <si>
-    <t>Asset is allocated with correct serial key syntax.</t>
-  </si>
-  <si>
-    <t>As Expected: Successfully allocated asset with matching corporate serial pattern.</t>
+    <t>Validate leave request requires all fields</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open Request Time Off modal.
+2. Click Submit without filling dates or reason.
+3. Verify required fields warning is shown.</t>
+  </si>
+  <si>
+    <t>Dates: blank | Reason: blank</t>
+  </si>
+  <si>
+    <t>Form displays error 'All fields are required.'.</t>
+  </si>
+  <si>
+    <t>As Expected: Submit blocked with required fields warning.</t>
   </si>
   <si>
     <t>TC#19</t>
   </si>
   <si>
-    <t>Track ticket status updates from Open to Resolved</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. File a support ticket.
-2. Admin resolves the ticket.
-3. Verify status field changes to 'Resolved'.</t>
-  </si>
-  <si>
-    <t>Ticket ID: 'tkt_502', Action: 'Resolve'</t>
-  </si>
-  <si>
-    <t>Ticket status updates from Open to Resolved.</t>
-  </si>
-  <si>
-    <t>As Expected: Ticket transition status changed to Resolved.</t>
+    <t>Validate empty announcement form block</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open Announcements Board.
+2. Click Publish without entering title or content.
+3. Verify submit is blocked (fields remain visible).</t>
+  </si>
+  <si>
+    <t>Title: blank | Content: blank</t>
+  </si>
+  <si>
+    <t>Form submission is blocked for empty announcement notice.</t>
+  </si>
+  <si>
+    <t>As Expected: Empty announcement publication blocked successfully.</t>
   </si>
   <si>
     <t>TC#20</t>
   </si>
   <si>
-    <t>Calculate corporate training compliance rate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Log completion count for GDPR training.
-2. Verify compliance percentage calculation accuracy.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> GDPR Course: Completed = 16, Total = 20</t>
-  </si>
-  <si>
-    <t>GDPR compliance percentage calculated to 80%.</t>
-  </si>
-  <si>
-    <t>As Expected: Compliance completion rate matches 80%.</t>
+    <t>Navigate to IT Assets page and verify inventory loads</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to IT Assets Admin in sidebar.
+2. Confirm total and active assets KPI counters display.
+3. Confirm asset inventory roster table loads rows.</t>
+  </si>
+  <si>
+    <t>Asset count KPIs</t>
+  </si>
+  <si>
+    <t>Hardware inventory details load and display in active asset dashboard.</t>
+  </si>
+  <si>
+    <t>As Expected: IT Assets dashboard loaded and displayed hardware roster table.</t>
+  </si>
+  <si>
+    <t>TC#21</t>
+  </si>
+  <si>
+    <t>Approve hardware request and verify active asset deployment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to IT Assets Admin.
+2. Locate pending request, click 'Approve &amp; Deploy'.
+3. Verify status becomes Approved and active assets count increases by 1.</t>
+  </si>
+  <si>
+    <t>Hardware Request: Monitor</t>
+  </si>
+  <si>
+    <t>Active asset count increases and deployment status updates.</t>
+  </si>
+  <si>
+    <t>As Expected: Request approved and active hardware inventory count increased by 1.</t>
+  </si>
+  <si>
+    <t>TC#22</t>
+  </si>
+  <si>
+    <t>Reject hardware request and verify request status changes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to IT Assets Admin.
+2. Locate pending request, click 'Reject'.
+3. Verify request status changes to Rejected.</t>
+  </si>
+  <si>
+    <t>Hardware Request: Laptop</t>
+  </si>
+  <si>
+    <t>Status badge updates to Rejected and request is completed.</t>
+  </si>
+  <si>
+    <t>As Expected: Hardware request rejected and status updated successfully.</t>
+  </si>
+  <si>
+    <t>TC#23</t>
+  </si>
+  <si>
+    <t>Navigate to Helpdesk page and verify tickets load</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to Helpdesk Tickets in sidebar.
+2. Verify open and resolved KPI cards are visible.
+3. Confirm ticket cards show in container.</t>
+  </si>
+  <si>
+    <t>Helpdesk support cards</t>
+  </si>
+  <si>
+    <t>Support ticket list populated with tickets and statistics.</t>
+  </si>
+  <si>
+    <t>As Expected: Helpdesk dashboard loaded ticket cards and resolved counts.</t>
+  </si>
+  <si>
+    <t>TC#24</t>
+  </si>
+  <si>
+    <t>Resolve open ticket and verify KPI status changes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to Helpdesk Tickets.
+2. Locate open ticket, click 'Resolve'.
+3. Verify open tickets count decreases by 1 and resolved count increases by 1.</t>
+  </si>
+  <si>
+    <t>Resolve Action: Open -&gt; Resolved</t>
+  </si>
+  <si>
+    <t>KPI counts adjust and ticket changes status indicator to Resolved.</t>
+  </si>
+  <si>
+    <t>As Expected: Ticket resolved and helpdesk statistics updated.</t>
+  </si>
+  <si>
+    <t>TC#25</t>
+  </si>
+  <si>
+    <t>Create new helpdesk ticket and verify in active roster</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to Helpdesk Tickets.
+2. Click 'New Ticket' to open form.
+3. Fill employee name, title, category, priority, and description.
+4. Click Submit, verify new ticket card displays in roster.</t>
+  </si>
+  <si>
+    <t>Title: E2E Selenium Test Ticket | Priority: Medium</t>
+  </si>
+  <si>
+    <t>New ticket submits successfully and shows up in cards list.</t>
+  </si>
+  <si>
+    <t>As Expected: Support ticket submitted and verified in active roster feed.</t>
+  </si>
+  <si>
+    <t>TC#26</t>
+  </si>
+  <si>
+    <t>Filter helpdesk tickets by status selection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to Helpdesk Tickets.
+2. Click 'Open' filter pill, verify only Open tickets are shown.
+3. Click 'Resolved' filter pill, verify only Resolved tickets are shown.</t>
+  </si>
+  <si>
+    <t>Filters: Open / Resolved</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Roster filters cards to only display selected ticket status.</t>
+  </si>
+  <si>
+    <t>As Expected: Ticket status filters successfully isolated Open and Resolved cases.</t>
   </si>
 </sst>
 </file>
@@ -909,7 +1051,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1007,7 +1149,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" ht="80" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>22</v>
       </c>
@@ -1030,7 +1172,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>29</v>
       </c>
@@ -1053,7 +1195,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" ht="80" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>35</v>
       </c>
@@ -1073,211 +1215,211 @@
         <v>40</v>
       </c>
       <c r="G13" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" ht="66" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="14" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+      <c r="B14" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="C14" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="D14" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="E14" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="F14" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="G14" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="G14" s="7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="15" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+      <c r="B15" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="C15" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="D15" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="E15" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="F15" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="G15" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" ht="66" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="G15" s="7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="16" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
+      <c r="B16" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="C16" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="D16" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="E16" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="F16" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="G16" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="G16" s="7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="17" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+      <c r="B17" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="C17" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="D17" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="E17" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="F17" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="G17" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" ht="80" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="G17" s="7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="18" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="5" t="s">
+      <c r="B18" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="C18" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="D18" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="E18" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="F18" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="G18" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" ht="80" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="G18" s="7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="19" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
+      <c r="B19" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="C19" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="D19" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="E19" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="F19" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="G19" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="G19" s="7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="20" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
+      <c r="B20" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="C20" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="D20" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="E20" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="F20" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="F20" s="6" t="s">
+      <c r="G20" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="21" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="G20" s="7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="21" ht="66" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
+      <c r="B21" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="C21" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="D21" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="E21" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="F21" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="G21" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="G21" s="7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="22" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="5" t="s">
+      <c r="B22" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="C22" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="D22" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="E22" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="F22" s="6" t="s">
         <v>94</v>
-      </c>
-      <c r="F22" s="6" t="s">
-        <v>95</v>
       </c>
       <c r="G22" s="7" t="s">
         <v>28</v>
@@ -1285,42 +1427,42 @@
     </row>
     <row r="23" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="C23" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="D23" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="E23" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="F23" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="G23" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="G23" s="7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="24" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="5" t="s">
+      <c r="B24" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="C24" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="D24" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="E24" s="6" t="s">
         <v>105</v>
-      </c>
-      <c r="E24" s="6" t="s">
-        <v>39</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>106</v>
@@ -1352,7 +1494,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="26" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>113</v>
       </c>
@@ -1375,7 +1517,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="27" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>119</v>
       </c>
@@ -1398,7 +1540,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="28" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>125</v>
       </c>
@@ -1444,7 +1586,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>137</v>
       </c>
@@ -1464,6 +1606,144 @@
         <v>142</v>
       </c>
       <c r="G30" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="31" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="G31" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="32" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="G32" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="33" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="G33" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="34" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="G34" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="35" ht="66" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="G35" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="36" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="G36" s="7" t="s">
         <v>28</v>
       </c>
     </row>

</xml_diff>